<commit_message>
Corrige skewness (bootstrap) no notebook 03 e comparacao WMT vs SPY no notebook 02
Notebook 03:
- o skewtest assume caudas normais e rejeita demasiado com curtose alta;
  a decisao do facto 3 passa a usar um bootstrap (IC 95% e p unilateral).
  Resultado: skewness negativa so significativa na frequencia semanal.
- texto do efeito alavanca menciona os modelos GARCH degenerados
- CSV gravados em utf-8-sig (Excel mostra bem os simbolos)
- exportado tambem em HTML

Notebook 02 (celula 36):
- comparava a WMT (com dividendos) com o ^GSPC (indice sem dividendos)
  chamado 'S&P 500'; agora mostra WMT, SPY (investivel) e ^GSPC
  com etiquetas claras, e seleciona as colunas antes do dropna

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011Eb8JJ3W1j7qqDmz3EZtgQ
</commit_message>
<xml_diff>
--- a/resultados/03_factos_estilizados.xlsx
+++ b/resultados/03_factos_estilizados.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="113">
   <si>
     <t>N</t>
   </si>
@@ -126,7 +126,16 @@
     <t>% |z|&gt;3 (normal)</t>
   </si>
   <si>
-    <t>Skew test stat</t>
+    <t>Skewtest p (assumes normal tails)</t>
+  </si>
+  <si>
+    <t>Bootstrap 95% CI low</t>
+  </si>
+  <si>
+    <t>Bootstrap 95% CI high</t>
+  </si>
+  <si>
+    <t>Bootstrap p (skew &gt;= 0)</t>
   </si>
   <si>
     <t>N below -3σ</t>
@@ -348,10 +357,10 @@
     <t>Supported</t>
   </si>
   <si>
+    <t>Not significant</t>
+  </si>
+  <si>
     <t>Partial</t>
-  </si>
-  <si>
-    <t>Not significant</t>
   </si>
   <si>
     <t>Not supported</t>
@@ -942,10 +951,10 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="B1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -1054,16 +1063,16 @@
         <v>10</v>
       </c>
       <c r="D1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F1" t="s">
         <v>19</v>
       </c>
       <c r="G1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -1077,16 +1086,16 @@
         <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F2">
         <v>0.001129726450990991</v>
       </c>
       <c r="G2" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -1100,16 +1109,16 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F3">
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -1123,16 +1132,16 @@
         <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F4">
-        <v>3.031500697858865E-11</v>
+        <v>0.2725</v>
       </c>
       <c r="G4" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -1146,16 +1155,16 @@
         <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F5">
         <v>5.328992409132081E-68</v>
       </c>
       <c r="G5" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -1169,16 +1178,16 @@
         <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E6" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F6">
         <v>0.00551755900227413</v>
       </c>
       <c r="G6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -1192,16 +1201,16 @@
         <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E7" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F7">
         <v>0</v>
       </c>
       <c r="G7" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -1215,16 +1224,16 @@
         <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E8" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F8">
         <v>0.1406127269999187</v>
       </c>
       <c r="G8" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -1238,16 +1247,16 @@
         <v>14</v>
       </c>
       <c r="D9" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E9" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="G9" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -1261,16 +1270,16 @@
         <v>14</v>
       </c>
       <c r="D10" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E10" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F10">
-        <v>1.091481970500465E-19</v>
+        <v>0.0265</v>
       </c>
       <c r="G10" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -1284,16 +1293,16 @@
         <v>14</v>
       </c>
       <c r="D11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E11" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F11">
         <v>0.1879552268363384</v>
       </c>
       <c r="G11" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -1307,16 +1316,16 @@
         <v>14</v>
       </c>
       <c r="D12" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="F12">
         <v>0.9787617727148507</v>
       </c>
       <c r="G12" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -1330,16 +1339,16 @@
         <v>14</v>
       </c>
       <c r="D13" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E13" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="F13">
         <v>0</v>
       </c>
       <c r="G13" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -1353,16 +1362,16 @@
         <v>15</v>
       </c>
       <c r="D14" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E14" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="F14">
         <v>0.6583005794510361</v>
       </c>
       <c r="G14" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -1376,16 +1385,16 @@
         <v>15</v>
       </c>
       <c r="D15" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E15" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F15">
         <v>0.006325960920331514</v>
       </c>
       <c r="G15" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -1399,16 +1408,16 @@
         <v>15</v>
       </c>
       <c r="D16" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E16" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="F16">
-        <v>0.03673840076158204</v>
+        <v>0.083</v>
       </c>
       <c r="G16" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -1422,16 +1431,16 @@
         <v>15</v>
       </c>
       <c r="D17" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E17" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F17">
         <v>0.6721661569493127</v>
       </c>
       <c r="G17" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -1445,16 +1454,16 @@
         <v>15</v>
       </c>
       <c r="D18" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E18" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="F18">
         <v>0.9999999893588277</v>
       </c>
       <c r="G18" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -1468,16 +1477,16 @@
         <v>15</v>
       </c>
       <c r="D19" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E19" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F19">
         <v>0.02865995652285228</v>
       </c>
       <c r="G19" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -1491,16 +1500,16 @@
         <v>13</v>
       </c>
       <c r="D20" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E20" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="F20">
         <v>6.557045906356267E-31</v>
       </c>
       <c r="G20" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -1514,16 +1523,16 @@
         <v>13</v>
       </c>
       <c r="D21" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E21" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F21">
         <v>0</v>
       </c>
       <c r="G21" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -1537,16 +1546,16 @@
         <v>13</v>
       </c>
       <c r="D22" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E22" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="F22">
-        <v>3.922231489479725E-43</v>
+        <v>0.113</v>
       </c>
       <c r="G22" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -1560,16 +1569,16 @@
         <v>13</v>
       </c>
       <c r="D23" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E23" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F23">
         <v>0</v>
       </c>
       <c r="G23" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1583,16 +1592,16 @@
         <v>13</v>
       </c>
       <c r="D24" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E24" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F24">
         <v>1.244520272204088E-17</v>
       </c>
       <c r="G24" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1606,16 +1615,16 @@
         <v>13</v>
       </c>
       <c r="D25" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E25" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="F25">
         <v>0</v>
       </c>
       <c r="G25" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1629,16 +1638,16 @@
         <v>14</v>
       </c>
       <c r="D26" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E26" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F26">
         <v>0.02378084994054098</v>
       </c>
       <c r="G26" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -1652,16 +1661,16 @@
         <v>14</v>
       </c>
       <c r="D27" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E27" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="F27">
         <v>1.193922935759543E-285</v>
       </c>
       <c r="G27" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -1675,16 +1684,16 @@
         <v>14</v>
       </c>
       <c r="D28" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E28" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="F28">
-        <v>6.019690746457557E-16</v>
+        <v>0.0285</v>
       </c>
       <c r="G28" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -1698,16 +1707,16 @@
         <v>14</v>
       </c>
       <c r="D29" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E29" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F29">
         <v>3.811664125226195E-79</v>
       </c>
       <c r="G29" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -1721,16 +1730,16 @@
         <v>14</v>
       </c>
       <c r="D30" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E30" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="F30">
         <v>1.911880780491605E-06</v>
       </c>
       <c r="G30" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -1744,16 +1753,16 @@
         <v>14</v>
       </c>
       <c r="D31" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E31" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="F31">
         <v>8.990624447866775E-67</v>
       </c>
       <c r="G31" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -1767,16 +1776,16 @@
         <v>15</v>
       </c>
       <c r="D32" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E32" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="F32">
         <v>0.2476046420882224</v>
       </c>
       <c r="G32" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -1790,16 +1799,16 @@
         <v>15</v>
       </c>
       <c r="D33" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E33" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="F33">
         <v>0.002854840932902221</v>
       </c>
       <c r="G33" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -1813,16 +1822,16 @@
         <v>15</v>
       </c>
       <c r="D34" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E34" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F34">
-        <v>0.005328155741619344</v>
+        <v>0.005</v>
       </c>
       <c r="G34" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -1836,16 +1845,16 @@
         <v>15</v>
       </c>
       <c r="D35" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E35" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="F35">
         <v>0.0005808780699925934</v>
       </c>
       <c r="G35" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -1859,16 +1868,16 @@
         <v>15</v>
       </c>
       <c r="D36" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E36" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F36">
         <v>0.5812759620288594</v>
       </c>
       <c r="G36" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -1882,16 +1891,16 @@
         <v>15</v>
       </c>
       <c r="D37" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E37" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="F37">
         <v>2.97550275901434E-05</v>
       </c>
       <c r="G37" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -1906,7 +1915,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B1" t="s">
         <v>13</v>
@@ -1920,86 +1929,86 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B2" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B4" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C4" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D4" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B5" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C5" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D5" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B6" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B7" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C7" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D7" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -2878,10 +2887,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>9</v>
       </c>
@@ -2895,22 +2904,28 @@
         <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
+        <v>38</v>
+      </c>
+      <c r="J1" t="s">
+        <v>39</v>
+      </c>
+      <c r="K1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -2921,25 +2936,31 @@
         <v>-0.2545877388259533</v>
       </c>
       <c r="D2">
-        <v>-6.645032551924453</v>
+        <v>3.031500697858865E-11</v>
       </c>
       <c r="E2">
-        <v>3.031500697858865E-11</v>
+        <v>-1.107911577087566</v>
       </c>
       <c r="F2">
+        <v>0.6029247587120391</v>
+      </c>
+      <c r="G2">
+        <v>0.2725</v>
+      </c>
+      <c r="H2">
         <v>30</v>
       </c>
-      <c r="G2">
+      <c r="I2">
         <v>28</v>
       </c>
-      <c r="H2">
+      <c r="J2">
         <v>-0.03253961619879404</v>
       </c>
-      <c r="I2">
+      <c r="K2">
         <v>0.03169501834639981</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:11">
       <c r="B3" t="s">
         <v>14</v>
       </c>
@@ -2947,25 +2968,31 @@
         <v>-0.853183233637098</v>
       </c>
       <c r="D3">
-        <v>-9.079426737612726</v>
+        <v>1.091481970500465E-19</v>
       </c>
       <c r="E3">
-        <v>1.091481970500465E-19</v>
+        <v>-1.768063409400142</v>
       </c>
       <c r="F3">
+        <v>0.002787724756609203</v>
+      </c>
+      <c r="G3">
+        <v>0.0265</v>
+      </c>
+      <c r="H3">
         <v>9</v>
       </c>
-      <c r="G3">
+      <c r="I3">
         <v>6</v>
       </c>
-      <c r="H3">
+      <c r="J3">
         <v>-0.07947422446551733</v>
       </c>
-      <c r="I3">
+      <c r="K3">
         <v>0.07668322868978676</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:11">
       <c r="B4" t="s">
         <v>15</v>
       </c>
@@ -2973,25 +3000,31 @@
         <v>-0.3602507848649407</v>
       </c>
       <c r="D4">
-        <v>-2.088659325158379</v>
+        <v>0.03673840076158204</v>
       </c>
       <c r="E4">
-        <v>0.03673840076158204</v>
+        <v>-0.7555658191388759</v>
       </c>
       <c r="F4">
+        <v>0.1454038441182619</v>
+      </c>
+      <c r="G4">
+        <v>0.083</v>
+      </c>
+      <c r="H4">
         <v>2</v>
       </c>
-      <c r="G4">
+      <c r="I4">
         <v>0</v>
       </c>
-      <c r="H4">
+      <c r="J4">
         <v>-0.129736763014624</v>
       </c>
-      <c r="I4">
+      <c r="K4">
         <v>0.1207657067668586</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:11">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -3002,25 +3035,31 @@
         <v>-0.5549130950810591</v>
       </c>
       <c r="D5">
-        <v>-13.76888438909523</v>
+        <v>3.922231489479725E-43</v>
       </c>
       <c r="E5">
-        <v>3.922231489479725E-43</v>
+        <v>-1.404203592831085</v>
       </c>
       <c r="F5">
+        <v>0.2771967688788283</v>
+      </c>
+      <c r="G5">
+        <v>0.113</v>
+      </c>
+      <c r="H5">
         <v>39</v>
       </c>
-      <c r="G5">
+      <c r="I5">
         <v>21</v>
       </c>
-      <c r="H5">
+      <c r="J5">
         <v>-0.03077065088726387</v>
       </c>
-      <c r="I5">
+      <c r="K5">
         <v>0.02605884237265368</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:11">
       <c r="B6" t="s">
         <v>14</v>
       </c>
@@ -3028,25 +3067,31 @@
         <v>-0.7400139267262549</v>
       </c>
       <c r="D6">
-        <v>-8.088918347514555</v>
+        <v>6.019690746457557E-16</v>
       </c>
       <c r="E6">
-        <v>6.019690746457557E-16</v>
+        <v>-1.51046699292638</v>
       </c>
       <c r="F6">
+        <v>0.0144957087309692</v>
+      </c>
+      <c r="G6">
+        <v>0.0285</v>
+      </c>
+      <c r="H6">
         <v>8</v>
       </c>
-      <c r="G6">
+      <c r="I6">
         <v>4</v>
       </c>
-      <c r="H6">
+      <c r="J6">
         <v>-0.06049433729176938</v>
       </c>
-      <c r="I6">
+      <c r="K6">
         <v>0.05693710518121</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:11">
       <c r="B7" t="s">
         <v>15</v>
       </c>
@@ -3054,21 +3099,27 @@
         <v>-0.4908913173960534</v>
       </c>
       <c r="D7">
-        <v>-2.786494286154341</v>
+        <v>0.005328155741619344</v>
       </c>
       <c r="E7">
-        <v>0.005328155741619344</v>
+        <v>-0.8506875669576397</v>
       </c>
       <c r="F7">
+        <v>-0.1117132724048969</v>
+      </c>
+      <c r="G7">
+        <v>0.005</v>
+      </c>
+      <c r="H7">
         <v>1</v>
       </c>
-      <c r="G7">
+      <c r="I7">
         <v>0</v>
       </c>
-      <c r="H7">
+      <c r="J7">
         <v>-0.0922649561467736</v>
       </c>
-      <c r="I7">
+      <c r="K7">
         <v>0.1032643850572533</v>
       </c>
     </row>
@@ -3097,16 +3148,16 @@
         <v>17</v>
       </c>
       <c r="D1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="G1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -3251,7 +3302,7 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B1" t="s">
         <v>11</v>
@@ -3388,37 +3439,37 @@
         <v>10</v>
       </c>
       <c r="C1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H1" t="s">
+        <v>50</v>
+      </c>
+      <c r="I1" t="s">
+        <v>51</v>
+      </c>
+      <c r="J1" t="s">
+        <v>52</v>
+      </c>
+      <c r="K1" t="s">
         <v>53</v>
       </c>
-      <c r="D1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F1" t="s">
-        <v>45</v>
-      </c>
-      <c r="G1" t="s">
-        <v>46</v>
-      </c>
-      <c r="H1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I1" t="s">
-        <v>48</v>
-      </c>
-      <c r="J1" t="s">
-        <v>49</v>
-      </c>
-      <c r="K1" t="s">
-        <v>50</v>
-      </c>
       <c r="L1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="M1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:13">
@@ -3429,7 +3480,7 @@
         <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D2">
         <v>0.1425185705710778</v>
@@ -3461,7 +3512,7 @@
     </row>
     <row r="3" spans="1:13">
       <c r="C3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D3">
         <v>0.1189639393732214</v>
@@ -3499,7 +3550,7 @@
         <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D4">
         <v>0.02263569615908406</v>
@@ -3531,7 +3582,7 @@
     </row>
     <row r="5" spans="1:13">
       <c r="C5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D5">
         <v>0.3157956082440811</v>
@@ -3569,7 +3620,7 @@
         <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D6">
         <v>3.054342150894797</v>
@@ -3601,7 +3652,7 @@
     </row>
     <row r="7" spans="1:13">
       <c r="C7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D7">
         <v>0.08715388417096093</v>
@@ -3642,7 +3693,7 @@
         <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D8">
         <v>0.03797816752193574</v>
@@ -3674,7 +3725,7 @@
     </row>
     <row r="9" spans="1:13">
       <c r="C9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D9">
         <v>0.02937232694013922</v>
@@ -3712,7 +3763,7 @@
         <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D10">
         <v>0.4711779154403531</v>
@@ -3744,7 +3795,7 @@
     </row>
     <row r="11" spans="1:13">
       <c r="C11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D11">
         <v>0.4258676091724037</v>
@@ -3782,7 +3833,7 @@
         <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D12">
         <v>4.537126524957438</v>
@@ -3814,7 +3865,7 @@
     </row>
     <row r="13" spans="1:13">
       <c r="C13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D13">
         <v>4.493564465168793</v>
@@ -3875,22 +3926,22 @@
         <v>10</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="G1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="H1" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -3901,7 +3952,7 @@
         <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D2">
         <v>-0.6435178675514044</v>
@@ -3921,7 +3972,7 @@
     </row>
     <row r="3" spans="1:8">
       <c r="C3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D3">
         <v>-0.6617199773355849</v>
@@ -3944,7 +3995,7 @@
         <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D4">
         <v>-0.783702699713868</v>
@@ -3964,7 +4015,7 @@
     </row>
     <row r="5" spans="1:8">
       <c r="C5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D5">
         <v>-0.994474851855187</v>
@@ -3987,7 +4038,7 @@
         <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D6">
         <v>-0.2505256480222186</v>
@@ -4007,7 +4058,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="C7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D7">
         <v>-0.3228412954318697</v>
@@ -4033,7 +4084,7 @@
         <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D8">
         <v>-0.7294045957934161</v>
@@ -4053,7 +4104,7 @@
     </row>
     <row r="9" spans="1:8">
       <c r="C9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D9">
         <v>-0.7943565750138284</v>
@@ -4076,7 +4127,7 @@
         <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D10">
         <v>-0.8441139367228159</v>
@@ -4096,7 +4147,7 @@
     </row>
     <row r="11" spans="1:8">
       <c r="C11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D11">
         <v>-0.8504013433396735</v>
@@ -4119,7 +4170,7 @@
         <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D12">
         <v>-0.753335971060093</v>
@@ -4139,7 +4190,7 @@
     </row>
     <row r="13" spans="1:8">
       <c r="C13" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D13">
         <v>-0.7751511297908221</v>

</xml_diff>